<commit_message>
Tracker: three rails measured, roadmap phases
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/AVNIHUB_TRACKER.xlsx
+++ b/docs/AVNIHUB_TRACKER.xlsx
@@ -417,14 +417,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="110" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="120" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -457,7 +457,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Project scaffold: 18 - Avni Vercel under AE Brain</t>
+          <t>Rename Avni Vercel -&gt; AvniHub (folders, engine, launcher, catalogue, repo)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -467,7 +467,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2 min</t>
+          <t>20 min</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -477,14 +477,14 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Canonical path D:\AE Brain\01 - Projects\18 - Avni Vercel\avni-vercel</t>
+          <t>01-09-2026 19:53. DB preserved through rename (submission 1 intact)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Engine avni_vercel.py: init/deploy/serve/submissions/export, SQLite-backed</t>
+          <t>Local rail: engine avnihub.py on :8190 (SQLite)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -494,7 +494,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>25 min</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -504,14 +504,14 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Stdlib only, port 8190, 10 MB upload cap, admin endpoints localhost-only</t>
+          <t>MEASURED 19:53: /health -&gt; AvniHub 0.1, sites 1, pages 2, submissions 1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Seed site sehgal-care (index.html + thanks.html)</t>
+          <t>Supabase master rail: avnihub_submissions + avnihub-receipts bucket + edge fn</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -521,7 +521,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>10 min</t>
+          <t>40 min</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -531,14 +531,14 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Sonnet worker card AV-18-001, reviewed, doctype defect corrected by Claude</t>
+          <t>MEASURED: public POST -&gt; ok id 1&amp;2; RLS ON, anon read = []; receipts in private bucket; project Sehgal Hero ap-south-1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>End-to-end verification: GET page, POST multipart, 303-&gt;thanks, DB row, export</t>
+          <t>Public page rail: GitHub Pages</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -548,7 +548,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5 min</t>
+          <t>15 min</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -558,14 +558,14 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>MEASURED 01-09-2026 18:57: submission id 1 stored; sha256 round-trip identical (6b7fa434...)</t>
+          <t>MEASURED: https://sehgalautoriders.github.io/avnihub/ -&gt; 200; page posts to edge fn; CORS verified from github.io origin</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LAN serving on 0.0.0.0:8190</t>
+          <t>GitHub repo sehgalautoriders/avnihub (public)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -585,19 +585,19 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>MEASURED: http://192.168.2.16:8190/sehgal-care/ -&gt; 200 from this PC</t>
+          <t>main cd44df1 + gh-pages branch; data/ git-ignored, no secrets in repo</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Phone-on-same-WiFi access</t>
+          <t>ROADMAP.md: all 21 Vercel uses mapped, phases v0.2-v0.6</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -607,19 +607,19 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1 click</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CONFIGURED - UNVERIFIED. No inbound firewall rule for 8190; Ravi runs 'Allow Avni Vercel on Wi-Fi.cmd' as admin</t>
+          <t>3 uses HAVE already (static hosting, CLI deploy, form capture - the last one Vercel itself lacks)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Public HTTPS URL for WhatsApp buttons</t>
+          <t>Phone-on-same-WiFi (local rail)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -634,19 +634,19 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Architect gate</t>
+          <t>1 click</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Internet-reach pillar: needs Architect + security review. Options: Cloudflare Tunnel from PC / Vercel Pro (paid, ToS-clean) / Supabase hosting. Vercel FREE tier prohibits commercial use - verified via web search 01-09-2026</t>
+          <t>Ravi: run 'Allow AvniHub on Wi-Fi.cmd' (Desktop) as administrator. NOTE: phones can already use the PUBLIC page instead</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Durable auto-start of server (survives session/reboot)</t>
+          <t>Own domain (avnihub.??)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -661,19 +661,19 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>15 min</t>
+          <t>days</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Session server running now; needs scheduled task or WMI launch + Store launch entry</t>
+          <t>Ravi: 'move to our own domain in some days'. Needs domain purchase (Ravi) + DNS + Pages custom domain + cert (auto)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Native tabbed admin UI (UI law)</t>
+          <t>v0.2: versioned deploys + rollback + request logs</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -688,19 +688,19 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>later</t>
+          <t>next</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>MVP admin = JSON endpoints + CLI; window owed per UI law</t>
+          <t>First build phase</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Supabase (One Brain) sync of submissions</t>
+          <t>Engine sync SQLite &lt;-&gt; Supabase (one command)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -720,24 +720,24 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Schema is lift-ready; do after pilot proves volume</t>
+          <t>Both rails live; sync closes the loop</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Avni Store catalogue row</t>
+          <t>WABA template -&gt; our URL</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2 min</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -747,19 +747,19 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Appended to avni-catalogue.json + .tsv, honest state</t>
+          <t>Public URL now EXISTS (github.io). Repoint = Meta re-approval; current leg on original Vercel via Antigravity - verify tier is commercial-compliant</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Git commit + push (AEBrain repo)</t>
+          <t>Trademark 'Avni' (lawyer)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Cannot do</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -769,24 +769,24 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Ravi</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Explicit paths only, no git add -A</t>
+          <t>Ravi's action with lawyer. Claude can prepare the brief: classes 9+42, ipindia prior-mark search</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>WABA template pointing at our own URL</t>
+          <t>Avni Store row (AvniHub)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Cannot do</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -801,7 +801,34 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Blocked until public-HTTPS decision; current approved template points at sehgal-care.vercel.app</t>
+          <t>Catalogue regenerated: 60 products, launcher rebuilt 50,688 B, payload staged</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Target: 1 year, 5000 apps, market entry</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>01-09-2027</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>~250 GB at 50 MB avg/app; storage pricing due at v0.4; tenant isolation + abuse controls before market</t>
         </is>
       </c>
     </row>

</xml_diff>